<commit_message>
Charge ambiguous tolls and fall back to date-overlap matching
Co-Authored-By: Amplify Shopify <amplifyonshopify@gmail.com>
</commit_message>
<xml_diff>
--- a/samples/turo_trips.xlsx
+++ b/samples/turo_trips.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,6 +560,33 @@
       <c r="E5" t="inlineStr">
         <is>
           <t>2026-03-15 12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>R-1005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Sam Lee</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Taofeek's Kia (GA #PLT9900)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-03-05 08:00</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-03-07 08:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Subtract Turo's Tolls & tickets charge from what the guest owes
Co-Authored-By: Amplify Shopify <amplifyonshopify@gmail.com>
</commit_message>
<xml_diff>
--- a/samples/turo_trips.xlsx
+++ b/samples/turo_trips.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,6 +454,11 @@
           <t>Trip end</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Tolls &amp; tickets</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -481,6 +486,11 @@
           <t>2026-03-03 11:00</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>$10.00</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -508,6 +518,7 @@
           <t>2026-03-06 18:00</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -535,6 +546,7 @@
           <t>2026-03-10 10:00</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -562,6 +574,7 @@
           <t>2026-03-15 12:00</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -589,6 +602,7 @@
           <t>2026-03-07 08:00</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Keep Turo-collected trips in What to charge even with no matched toll
Co-Authored-By: Amplify Shopify <amplifyonshopify@gmail.com>
</commit_message>
<xml_diff>
--- a/samples/turo_trips.xlsx
+++ b/samples/turo_trips.xlsx
@@ -602,7 +602,11 @@
           <t>2026-03-07 08:00</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>$4.00</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>